<commit_message>
App: Registro asistencia - ARTES PLÁSTICAS
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -898,6 +898,386 @@
         <v>1</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ARTES PLÁSTICAS</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
App: Registro asistencia - ARTE Y PINTURA
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1938,6 +1938,346 @@
         <v>1.5</v>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>ARTE Y PINTURA</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
App: Registro asistencia - ACTIVIDAD FÍSICA Y DEPORTE
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D93"/>
+  <dimension ref="A1:D112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2278,6 +2278,386 @@
         <v>3.25</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>JESÚS SALCIDO ZAMORA</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Admin: Eliminación de 5 registros individuales del día 19/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D112"/>
+  <dimension ref="A1:D107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1521,12 +1521,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1541,12 +1541,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1561,12 +1561,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1581,12 +1581,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1601,12 +1601,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1846,16 +1846,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="73">
@@ -1866,16 +1866,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="74">
@@ -1886,16 +1886,16 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="75">
@@ -1906,16 +1906,16 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="76">
@@ -1926,16 +1926,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="77">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2181,101 +2181,101 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2506,7 +2506,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -2555,106 +2555,6 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D108" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D109" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D110" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D111" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D112" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin: Eliminación de 2 registros individuales del día 20/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D107"/>
+  <dimension ref="A1:D105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -686,7 +686,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -866,16 +866,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -886,16 +886,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -906,7 +906,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1241,12 +1241,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1255,18 +1255,18 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="44">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1481,12 +1481,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1501,12 +1501,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1806,16 +1806,16 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="71">
@@ -1826,16 +1826,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="72">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2141,41 +2141,41 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2506,7 +2506,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2515,46 +2515,6 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D106" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D107" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin: Eliminación de 5 registros individuales del día 20/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D105"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -686,7 +686,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -826,16 +826,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -846,16 +846,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -866,7 +866,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1201,12 +1201,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1215,18 +1215,18 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="42">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1441,12 +1441,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1461,12 +1461,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1766,16 +1766,16 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="69">
@@ -1786,16 +1786,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="70">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2101,41 +2101,41 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2415,106 +2415,6 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D101" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D102" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D103" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D104" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D105" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin: Eliminación de 8 registros individuales del día 20/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D93"/>
+  <dimension ref="A1:D85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2118,166 +2118,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D86" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D87" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D88" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D89" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D90" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D91" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D92" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D93" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Admin: Eliminación de 12 registros individuales del día 20/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -546,16 +546,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -566,16 +566,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -586,16 +586,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -606,16 +606,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -626,16 +626,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -646,16 +646,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -666,16 +666,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -686,16 +686,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -706,16 +706,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -726,16 +726,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -746,16 +746,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -766,16 +766,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -786,7 +786,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -921,12 +921,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -935,18 +935,18 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -955,18 +955,18 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -975,18 +975,18 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -995,18 +995,18 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1015,18 +1015,18 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1035,18 +1035,18 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1055,18 +1055,18 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1075,18 +1075,18 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1095,18 +1095,18 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1115,18 +1115,18 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1135,18 +1135,18 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1155,13 +1155,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1181,7 +1181,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1201,7 +1201,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1221,7 +1221,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1261,7 +1261,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1281,7 +1281,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1301,7 +1301,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1321,7 +1321,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1341,12 +1341,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1361,12 +1361,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1381,12 +1381,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1486,16 +1486,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="55">
@@ -1506,16 +1506,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="56">
@@ -1526,16 +1526,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="57">
@@ -1546,16 +1546,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="58">
@@ -1566,16 +1566,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="59">
@@ -1586,16 +1586,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="60">
@@ -1606,16 +1606,16 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="61">
@@ -1626,16 +1626,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="62">
@@ -1646,16 +1646,16 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="63">
@@ -1666,16 +1666,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="64">
@@ -1686,16 +1686,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="65">
@@ -1706,16 +1706,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="66">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1821,300 +1821,60 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>16/05/2026</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D74" t="n">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>16/05/2026</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D75" t="n">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>16/05/2026</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D76" t="n">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>16/05/2026</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D77" t="n">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>16/05/2026</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D78" t="n">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>16/05/2026</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D79" t="n">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>16/05/2026</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D80" t="n">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>16/05/2026</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D81" t="n">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>16/05/2026</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D82" t="n">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D83" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D84" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D85" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin: Eliminación de 3 registros individuales del día 20/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1338,66 +1338,6 @@
         <v>3.25</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>20/05/2026</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD FÍSICA Y DEPORTE</t>
-        </is>
-      </c>
-      <c r="D49" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
App: Registro asistencia - COCINA Y REPOSTERÍA
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1618,6 +1618,226 @@
         <v>2</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>COCINA Y REPOSTERÍA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
App: Registro asistencia - CONVIVENCIA INSTITUCIONAL
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D134"/>
+  <dimension ref="A1:D157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3098,6 +3098,466 @@
         <v>2</v>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>JESÚS SALCIDO ZAMORA</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
App: Registro asistencia - AUTONOMÍA Y VIDA INDEPENDIENTE
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D157"/>
+  <dimension ref="A1:D180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3558,6 +3558,466 @@
         <v>1</v>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>JESÚS SALCIDO ZAMORA</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Admin: Eliminación de 2 registros individuales del día 22/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D249"/>
+  <dimension ref="A1:D247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -3886,7 +3886,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -3986,7 +3986,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -4066,7 +4066,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4086,7 +4086,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4106,7 +4106,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4126,7 +4126,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -4186,7 +4186,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -4286,7 +4286,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -4406,7 +4406,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -4466,7 +4466,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -4526,7 +4526,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -4566,7 +4566,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -4606,7 +4606,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -4626,7 +4626,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -4646,7 +4646,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -4686,7 +4686,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -4746,7 +4746,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -4846,7 +4846,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -4866,7 +4866,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -4901,41 +4901,41 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>22/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>2.25</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>22/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>2.25</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="227">
@@ -4946,7 +4946,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -4966,7 +4966,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -5046,7 +5046,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -5146,7 +5146,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -5226,7 +5226,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -5246,7 +5246,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -5266,7 +5266,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -5326,7 +5326,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -5355,46 +5355,6 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="B248" t="inlineStr">
-        <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
-        </is>
-      </c>
-      <c r="C248" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D248" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="B249" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C249" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D249" t="n">
         <v>1.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin: Eliminación de 1 registros individuales del día 22/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D181"/>
+  <dimension ref="A1:D180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3561,21 +3561,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>22/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>AUTONOMÍA Y VIDA INDEPENDIENTE</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>2.25</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="159">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -3886,7 +3886,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -3986,7 +3986,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -4015,26 +4015,6 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D181" t="n">
         <v>1.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin: Eliminación de 1 registros individuales del día 21/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D180"/>
+  <dimension ref="A1:D179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -3886,7 +3886,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -3986,7 +3986,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -3995,26 +3995,6 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D180" t="n">
         <v>1.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin: Eliminación de 2 registros individuales del día 21/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D159"/>
+  <dimension ref="A1:D157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3558,46 +3558,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D158" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>ARTE Y PINTURA</t>
-        </is>
-      </c>
-      <c r="D159" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Asistencia: Registro real de GRUPO DE CRECIMIENTO - 26/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D157"/>
+  <dimension ref="A1:D163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3558,6 +3558,126 @@
         <v>1</v>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>JESÚS SALCIDO ZAMORA</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Asistencia: Registro Directo de GRUPO DE CRECIMIENTO - 22/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D163"/>
+  <dimension ref="A1:D180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3678,6 +3678,346 @@
         <v>1</v>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>JESÚS SALCIDO ZAMORA</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Asistencia: Registro real de GRUPO DE CRECIMIENTO (nan) - 26/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D180"/>
+  <dimension ref="A1:D191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4018,6 +4018,226 @@
         <v>2.25</v>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO (nan)</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO (nan)</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>JESÚS SALCIDO ZAMORA</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO (nan)</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO (nan)</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO (nan)</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO (nan)</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO (nan)</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO (nan)</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO (nan)</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO (nan)</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO (nan)</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Admin: Eliminación de 17 registros individuales del día 26/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D191"/>
+  <dimension ref="A1:D174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3561,7 +3561,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -3575,18 +3575,18 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -3595,18 +3595,18 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3615,18 +3615,18 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -3635,18 +3635,18 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -3655,18 +3655,18 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -3675,7 +3675,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="164">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -3886,7 +3886,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -3896,346 +3896,6 @@
       </c>
       <c r="D174" t="n">
         <v>2.25</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D175" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D176" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D177" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D178" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D179" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D180" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>26/05/2026</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO (nan)</t>
-        </is>
-      </c>
-      <c r="D181" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>26/05/2026</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO (nan)</t>
-        </is>
-      </c>
-      <c r="D182" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>26/05/2026</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO (nan)</t>
-        </is>
-      </c>
-      <c r="D183" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>26/05/2026</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO (nan)</t>
-        </is>
-      </c>
-      <c r="D184" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>26/05/2026</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO (nan)</t>
-        </is>
-      </c>
-      <c r="D185" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>26/05/2026</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO (nan)</t>
-        </is>
-      </c>
-      <c r="D186" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>26/05/2026</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO (nan)</t>
-        </is>
-      </c>
-      <c r="D187" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>26/05/2026</t>
-        </is>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
-        </is>
-      </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO (nan)</t>
-        </is>
-      </c>
-      <c r="D188" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>26/05/2026</t>
-        </is>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
-        </is>
-      </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO (nan)</t>
-        </is>
-      </c>
-      <c r="D189" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>26/05/2026</t>
-        </is>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO (nan)</t>
-        </is>
-      </c>
-      <c r="D190" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>26/05/2026</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO (nan)</t>
-        </is>
-      </c>
-      <c r="D191" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Admin: Eliminación de 6 registros individuales del día 22/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D174"/>
+  <dimension ref="A1:D168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -3775,126 +3775,6 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
-        </is>
-      </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D169" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
-        </is>
-      </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D170" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D171" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
-        </is>
-      </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D172" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D173" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D174" t="n">
         <v>2.25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin: Eliminación de 5 registros individuales del día 22/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D162"/>
+  <dimension ref="A1:D157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3558,106 +3558,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D158" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D159" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D160" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D161" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D162" t="n">
-        <v>2.25</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Admin: Borrado de 10 registros del 21/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D157"/>
+  <dimension ref="A1:D147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1641,201 +1641,201 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>COCINA Y REPOSTERÍA</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>COCINA Y REPOSTERÍA</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>COCINA Y REPOSTERÍA</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>COCINA Y REPOSTERÍA</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>COCINA Y REPOSTERÍA</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>COCINA Y REPOSTERÍA</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>COCINA Y REPOSTERÍA</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>COCINA Y REPOSTERÍA</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>COCINA Y REPOSTERÍA</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>COCINA Y REPOSTERÍA</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="72">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2441,201 +2441,201 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="112">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -2901,201 +2901,201 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -3355,206 +3355,6 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>CONVIVENCIA INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="D148" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>CONVIVENCIA INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="D149" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>CONVIVENCIA INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="D150" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>CONVIVENCIA INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="D151" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>CONVIVENCIA INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="D152" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>CONVIVENCIA INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="D153" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>CONVIVENCIA INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="D154" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>CONVIVENCIA INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="D155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>CONVIVENCIA INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="D156" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>CONVIVENCIA INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="D157" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin: Borrado de 1 registros del 21/05/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D147"/>
+  <dimension ref="A1:D146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1621,21 +1621,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>COCINA Y REPOSTERÍA</t>
+          <t>ARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="62">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2421,21 +2421,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ARTES PLÁSTICAS</t>
+          <t>ARTE Y PINTURA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="102">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2506,7 +2506,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2881,21 +2881,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>ARTE Y PINTURA</t>
+          <t>CONVIVENCIA INSTITUCIONAL</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>EFRAÍN MAYNEZ PORRAS</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>EFRAÍN MAYNEZ PORRAS</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>JESÚS SALCIDO ZAMORA</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>JESÚS SALCIDO ZAMORA</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -3335,26 +3335,6 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>19/05/2026</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>CONVIVENCIA INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="D147" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Asistencia: TALLER "SÍ PUEDO" (10:00 - 12:00)
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D146"/>
+  <dimension ref="A1:D153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3338,6 +3338,146 @@
         <v>1</v>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO" (10:00 - 12:00)</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO" (10:00 - 12:00)</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO" (10:00 - 12:00)</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO" (10:00 - 12:00)</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO" (10:00 - 12:00)</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO" (10:00 - 12:00)</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO" (10:00 - 12:00)</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Asistencia: DESARROLLO EDUCATIVO (09:00 - 10:30) el 09/07/2026
</commit_message>
<xml_diff>
--- a/asistencia.xlsx
+++ b/asistencia.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D426"/>
+  <dimension ref="A1:D431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8938,6 +8938,106 @@
         <v>1.5</v>
       </c>
     </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>DESARROLLO EDUCATIVO (09:00 - 10:30)</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>DESARROLLO EDUCATIVO (09:00 - 10:30)</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>DESARROLLO EDUCATIVO (09:00 - 10:30)</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>ISAAC IGNACIO GONZÁLEZ CRUZ</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>DESARROLLO EDUCATIVO (09:00 - 10:30)</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>JESÚS SALCIDO ZAMORA</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>DESARROLLO EDUCATIVO (09:00 - 10:30)</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>